<commit_message>
Continued Excel practice functions and updated documentation.
</commit_message>
<xml_diff>
--- a/excel/excel_job_search_practice.xlsx
+++ b/excel/excel_job_search_practice.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\defaultuser0\Documents\nicosys-da-gym\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{282C54C1-306B-43AE-9C9B-1FB9397B09CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C213B89-275A-4BE9-9AB9-880D0D49F719}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19110" yWindow="0" windowWidth="38580" windowHeight="10530" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25690" yWindow="2050" windowWidth="30810" windowHeight="9960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw_Data" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="96">
   <si>
     <t>Application_ID</t>
   </si>
@@ -320,6 +320,9 @@
   </si>
   <si>
     <t>Average values matching multiple conditions</t>
+  </si>
+  <si>
+    <t>Cout all applications with Status = "Rejected"</t>
   </si>
 </sst>
 </file>
@@ -433,7 +436,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -477,6 +480,14 @@
     <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -492,6 +503,23 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -711,10 +739,10 @@
   <cols>
     <col min="1" max="1" width="11.69921875" customWidth="1"/>
     <col min="2" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="7.59765625" customWidth="1"/>
-    <col min="5" max="5" width="9.09765625" customWidth="1"/>
-    <col min="6" max="6" width="9.5" customWidth="1"/>
-    <col min="7" max="7" width="8.19921875" customWidth="1"/>
+    <col min="4" max="4" width="7.8984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.8984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.3984375" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="22" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1169,13 +1197,15 @@
         <v>62</v>
       </c>
       <c r="D4" s="6">
-        <f>_xlfn.XLOOKUP("Mercury Insurance",Raw_Data!B:B, Raw_Data!F:F)</f>
+        <f>_xlfn.XLOOKUP("Mercury Insurance", JobSearch[Company], JobSearch[Salary_Max])</f>
         <v>80000</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="F4" s="2"/>
+      <c r="F4" s="17" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="2">
@@ -1194,7 +1224,9 @@
       <c r="E5" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="F5" s="2"/>
+      <c r="F5" s="17" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="2">
@@ -1213,7 +1245,9 @@
       <c r="E6" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="F6" s="2"/>
+      <c r="F6" s="17" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="2">
@@ -1232,7 +1266,9 @@
       <c r="E7" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="F7" s="2"/>
+      <c r="F7" s="17" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="2">
@@ -1244,11 +1280,16 @@
       <c r="C8" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="D8" s="7"/>
+      <c r="D8" s="7">
+        <f>AVERAGEIFS(JobSearch[Salary_Max], JobSearch[Status], "Interview", JobSearch[Fit_Rating], "&gt;=8")</f>
+        <v>71500</v>
+      </c>
       <c r="E8" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F8" s="2"/>
+      <c r="F8" s="17" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="2">
@@ -1260,11 +1301,16 @@
       <c r="C9" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D9" s="7"/>
+      <c r="D9" s="7">
+        <f>COUNTIFS(JobSearch[Status], "Interview", JobSearch[Fit_Rating], "&gt;=8")</f>
+        <v>4</v>
+      </c>
       <c r="E9" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F9" s="2"/>
+      <c r="F9" s="17" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="2">
@@ -1276,11 +1322,16 @@
       <c r="C10" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D10" s="7"/>
+      <c r="D10" s="7">
+        <f>SUMIFS(JobSearch[Salary_Max], JobSearch[Status], "Interview", JobSearch[Fit_Rating], "&gt;=8")</f>
+        <v>286000</v>
+      </c>
       <c r="E10" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F10" s="2"/>
+      <c r="F10" s="17" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="2">
@@ -1292,11 +1343,37 @@
       <c r="C11" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D11" s="8"/>
+      <c r="D11" s="8">
+        <f>COUNTIF(JobSearch[Status], "Applied")</f>
+        <v>4</v>
+      </c>
       <c r="E11" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="F11" s="2"/>
+      <c r="F11" s="17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="2">
+        <v>9</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D12">
+        <f>COUNTIF(JobSearch[Status], "Rejected")</f>
+        <v>3</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F12" s="17" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="14" t="s">

</xml_diff>